<commit_message>
Free tools carousel published (media 17955168417254149)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="15" min="1" max="1"/>
@@ -665,18 +665,18 @@
       </c>
     </row>
     <row r="5" ht="33.75" customHeight="1" s="16">
-      <c r="A5" s="20" t="n">
+      <c r="A5" s="23" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>46305</v>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>السبت</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>5:00 م</t>
         </is>
@@ -686,33 +686,33 @@
           <t>3 أدوات مجانية تغنيك عن المدفوعة</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G5" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="20" t="inlineStr">
-        <is>
-          <t>مجدول</t>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>منشور</t>
         </is>
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>الكابشن معتمد، وبيوصلك الرابط أول ما ينزل</t>
+          <t>نزل 5:17 العصر: https://www.instagram.com/p/DeT2Q92Fbv3/</t>
         </is>
       </c>
     </row>
     <row r="6" ht="33.75" customHeight="1" s="16">
-      <c r="A6" s="20" t="n">
+      <c r="A6" s="23" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>46306</v>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>الأحد</t>
         </is>
@@ -727,15 +727,15 @@
           <t>الشحن السريع للسيارة الكهربائية صار أغلى من البنزين</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="23" t="inlineStr">
         <is>
           <t>مجدول</t>
         </is>
@@ -747,24 +747,24 @@
       </c>
     </row>
     <row r="7" ht="33.75" customHeight="1" s="16">
-      <c r="A7" s="20" t="n">
+      <c r="A7" s="23" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="21" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="20" t="n"/>
+      <c r="C7" s="23" t="n"/>
+      <c r="D7" s="23" t="n"/>
       <c r="E7" s="22" t="inlineStr">
         <is>
           <t>ريل المنطقة الاقتصادية للذكاء الاصطناعي في عُمان (النسخة 8، الصوت الثاني)</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="23" t="inlineStr">
         <is>
           <t>ريل</t>
         </is>
       </c>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="G7" s="23" t="n"/>
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>جاهز</t>
         </is>
@@ -776,24 +776,24 @@
       </c>
     </row>
     <row r="8" ht="33.75" customHeight="1" s="16">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="23" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="21" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="23" t="n"/>
       <c r="E8" s="22" t="inlineStr">
         <is>
           <t>ملف خطة الـ30 ريل</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="23" t="inlineStr">
         <is>
           <t>ملف PDF</t>
         </is>
       </c>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="20" t="inlineStr">
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>جاهز</t>
         </is>
@@ -801,24 +801,24 @@
       <c r="I8" s="22" t="n"/>
     </row>
     <row r="9" ht="33.75" customHeight="1" s="16">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="21" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
+      <c r="C9" s="23" t="n"/>
+      <c r="D9" s="23" t="n"/>
       <c r="E9" s="22" t="inlineStr">
         <is>
           <t>مستند خطة الكاروسيلات السبعة</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="F9" s="23" t="inlineStr">
         <is>
           <t>مستند</t>
         </is>
       </c>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="inlineStr">
+      <c r="G9" s="23" t="n"/>
+      <c r="H9" s="23" t="inlineStr">
         <is>
           <t>جاهز</t>
         </is>
@@ -830,13 +830,13 @@
       </c>
     </row>
     <row r="10" ht="33.75" customHeight="1" s="16">
-      <c r="A10" s="20" t="n">
+      <c r="A10" s="23" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="21" t="n">
         <v>46307</v>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>الاثنين</t>
         </is>
@@ -851,13 +851,13 @@
           <t>سيارة بلا مقود</t>
         </is>
       </c>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="F10" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G10" s="20" t="n"/>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="G10" s="23" t="n"/>
+      <c r="H10" s="23" t="inlineStr">
         <is>
           <t>ما تصمّم</t>
         </is>
@@ -869,13 +869,13 @@
       </c>
     </row>
     <row r="11" ht="33.75" customHeight="1" s="16">
-      <c r="A11" s="20" t="n">
+      <c r="A11" s="23" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="21" t="n">
         <v>46308</v>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>الثلاثاء</t>
         </is>
@@ -890,13 +890,13 @@
           <t>المجاني بدأ ينكمش</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="20" t="inlineStr">
+      <c r="G11" s="23" t="n"/>
+      <c r="H11" s="23" t="inlineStr">
         <is>
           <t>ما تصمّم</t>
         </is>
@@ -908,13 +908,13 @@
       </c>
     </row>
     <row r="12" ht="33.75" customHeight="1" s="16">
-      <c r="A12" s="20" t="n">
+      <c r="A12" s="23" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="21" t="n">
         <v>46309</v>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>الأربعاء</t>
         </is>
@@ -929,13 +929,13 @@
           <t>500 مشروع درون (يعرّف فيك)</t>
         </is>
       </c>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="F12" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="20" t="inlineStr">
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="23" t="inlineStr">
         <is>
           <t>ما تصمّم</t>
         </is>
@@ -947,13 +947,13 @@
       </c>
     </row>
     <row r="13" ht="33.75" customHeight="1" s="16">
-      <c r="A13" s="20" t="n">
+      <c r="A13" s="23" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="21" t="n">
         <v>46310</v>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>الخميس</t>
         </is>
@@ -968,13 +968,13 @@
           <t>ذكاء اصطناعي يسوق معك</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F13" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="20" t="inlineStr">
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="23" t="inlineStr">
         <is>
           <t>ما تصمّم</t>
         </is>
@@ -986,13 +986,13 @@
       </c>
     </row>
     <row r="14" ht="33.75" customHeight="1" s="16">
-      <c r="A14" s="20" t="n">
+      <c r="A14" s="23" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="21" t="n">
         <v>46311</v>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>الجمعة</t>
         </is>
@@ -1007,13 +1007,13 @@
           <t>رسالة المخالفة فخ</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="20" t="inlineStr">
+      <c r="G14" s="23" t="n"/>
+      <c r="H14" s="23" t="inlineStr">
         <is>
           <t>ما تصمّم</t>
         </is>
@@ -1025,13 +1025,13 @@
       </c>
     </row>
     <row r="15" ht="33.75" customHeight="1" s="16">
-      <c r="A15" s="20" t="n">
+      <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="21" t="n">
         <v>46312</v>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>السبت</t>
         </is>
@@ -1046,13 +1046,13 @@
           <t>روبوت بسعر سيارة</t>
         </is>
       </c>
-      <c r="F15" s="20" t="inlineStr">
+      <c r="F15" s="23" t="inlineStr">
         <is>
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="inlineStr">
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="23" t="inlineStr">
         <is>
           <t>ما تصمّم</t>
         </is>
@@ -1063,6 +1063,8 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="E18" s="25" t="inlineStr">
         <is>
@@ -1143,6 +1145,20 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <autoFilter ref="A4:I15"/>
   <conditionalFormatting sqref="A5:I35">

</xml_diff>

<commit_message>
AI weekly roundup #1: 15 slides, caption and links page (manual publish)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="15" min="1" max="1"/>
@@ -617,6 +617,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="16">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -737,12 +738,12 @@
       </c>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>مجدول</t>
+          <t>منشور</t>
         </is>
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>اليوم 1 من خطة الأسبوع، وبيوصلك الرابط أول ما ينزل</t>
+          <t>نزل 5:04 العصر: https://www.instagram.com/p/DeWuREyDGWc/</t>
         </is>
       </c>
     </row>
@@ -848,7 +849,7 @@
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>سيارة بلا مقود</t>
+          <t>ملخص أسبوع الذكاء الاصطناعي (العدد 1)</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
@@ -856,15 +857,17 @@
           <t>كاروسل</t>
         </is>
       </c>
-      <c r="G10" s="23" t="n"/>
+      <c r="G10" s="23" t="n">
+        <v>15</v>
+      </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>ما تصمّم</t>
+          <t>جاهز</t>
         </is>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>اليوم 2</t>
+          <t>زياد ينشره يدويًا 5 العصر (15 شريحة أكثر من حد النشر التلقائي). صفحة الروابط في البايو. "سيارة بلا مقود" تأجلت</t>
         </is>
       </c>
     </row>
@@ -1145,20 +1148,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <autoFilter ref="A4:I15"/>
   <conditionalFormatting sqref="A5:I35">

</xml_diff>

<commit_message>
Tracker: cancel the unapproved 7-carousel plan and its schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -613,11 +613,10 @@
     <row r="2" ht="15" customHeight="1" s="16">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>آخر تحديث: 10 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>آخر تحديث: 12 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="30" customHeight="1" s="16">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -805,20 +804,32 @@
       <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="23" t="n"/>
-      <c r="D9" s="23" t="n"/>
+      <c r="B9" s="21" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
       <c r="E9" s="22" t="inlineStr">
         <is>
-          <t>مستند خطة الكاروسيلات السبعة</t>
+          <t>ملخص أسبوع الذكاء الاصطناعي (العدد 1)</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>مستند</t>
-        </is>
-      </c>
-      <c r="G9" s="23" t="n"/>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>15</v>
+      </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
           <t>جاهز</t>
@@ -826,248 +837,76 @@
       </c>
       <c r="I9" s="24" t="inlineStr">
         <is>
-          <t>رابط المستند</t>
+          <t>زياد ينشره يدويًا 5 العصر (15 شريحة أكثر من حد النشر التلقائي). صفحة الروابط في البايو.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="33.75" customHeight="1" s="16">
-      <c r="A10" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <v>46307</v>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>الاثنين</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>5:00 م</t>
-        </is>
-      </c>
-      <c r="E10" s="22" t="inlineStr">
-        <is>
-          <t>ملخص أسبوع الذكاء الاصطناعي (العدد 1)</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>كاروسل</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="H10" s="23" t="inlineStr">
-        <is>
-          <t>جاهز</t>
-        </is>
-      </c>
-      <c r="I10" s="22" t="inlineStr">
-        <is>
-          <t>زياد ينشره يدويًا 5 العصر (15 شريحة أكثر من حد النشر التلقائي). صفحة الروابط في البايو. "سيارة بلا مقود" تأجلت</t>
-        </is>
-      </c>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="21" t="n"/>
+      <c r="C10" s="23" t="n"/>
+      <c r="D10" s="23" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="23" t="n"/>
+      <c r="G10" s="23" t="n"/>
+      <c r="H10" s="23" t="n"/>
+      <c r="I10" s="22" t="n"/>
     </row>
     <row r="11" ht="33.75" customHeight="1" s="16">
-      <c r="A11" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>46308</v>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>الثلاثاء</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>5:00 م</t>
-        </is>
-      </c>
-      <c r="E11" s="22" t="inlineStr">
-        <is>
-          <t>المجاني بدأ ينكمش</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
-        <is>
-          <t>كاروسل</t>
-        </is>
-      </c>
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="23" t="n"/>
+      <c r="D11" s="23" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="23" t="n"/>
       <c r="G11" s="23" t="n"/>
-      <c r="H11" s="23" t="inlineStr">
-        <is>
-          <t>ما تصمّم</t>
-        </is>
-      </c>
-      <c r="I11" s="22" t="inlineStr">
-        <is>
-          <t>اليوم 3</t>
-        </is>
-      </c>
+      <c r="H11" s="23" t="n"/>
+      <c r="I11" s="22" t="n"/>
     </row>
     <row r="12" ht="33.75" customHeight="1" s="16">
-      <c r="A12" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>46309</v>
-      </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>الأربعاء</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>5:00 م</t>
-        </is>
-      </c>
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>500 مشروع درون (يعرّف فيك)</t>
-        </is>
-      </c>
-      <c r="F12" s="23" t="inlineStr">
-        <is>
-          <t>كاروسل</t>
-        </is>
-      </c>
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="21" t="n"/>
+      <c r="C12" s="23" t="n"/>
+      <c r="D12" s="23" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="23" t="n"/>
       <c r="G12" s="23" t="n"/>
-      <c r="H12" s="23" t="inlineStr">
-        <is>
-          <t>ما تصمّم</t>
-        </is>
-      </c>
-      <c r="I12" s="22" t="inlineStr">
-        <is>
-          <t>اليوم 4</t>
-        </is>
-      </c>
+      <c r="H12" s="23" t="n"/>
+      <c r="I12" s="22" t="n"/>
     </row>
     <row r="13" ht="33.75" customHeight="1" s="16">
-      <c r="A13" s="23" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="21" t="n">
-        <v>46310</v>
-      </c>
-      <c r="C13" s="23" t="inlineStr">
-        <is>
-          <t>الخميس</t>
-        </is>
-      </c>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t>5:00 م</t>
-        </is>
-      </c>
-      <c r="E13" s="22" t="inlineStr">
-        <is>
-          <t>ذكاء اصطناعي يسوق معك</t>
-        </is>
-      </c>
-      <c r="F13" s="23" t="inlineStr">
-        <is>
-          <t>كاروسل</t>
-        </is>
-      </c>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="23" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="23" t="n"/>
       <c r="G13" s="23" t="n"/>
-      <c r="H13" s="23" t="inlineStr">
-        <is>
-          <t>ما تصمّم</t>
-        </is>
-      </c>
-      <c r="I13" s="22" t="inlineStr">
-        <is>
-          <t>اليوم 5</t>
-        </is>
-      </c>
+      <c r="H13" s="23" t="n"/>
+      <c r="I13" s="22" t="n"/>
     </row>
     <row r="14" ht="33.75" customHeight="1" s="16">
-      <c r="A14" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>46311</v>
-      </c>
-      <c r="C14" s="23" t="inlineStr">
-        <is>
-          <t>الجمعة</t>
-        </is>
-      </c>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>5:00 م</t>
-        </is>
-      </c>
-      <c r="E14" s="22" t="inlineStr">
-        <is>
-          <t>رسالة المخالفة فخ</t>
-        </is>
-      </c>
-      <c r="F14" s="23" t="inlineStr">
-        <is>
-          <t>كاروسل</t>
-        </is>
-      </c>
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="23" t="n"/>
+      <c r="D14" s="23" t="n"/>
+      <c r="E14" s="22" t="n"/>
+      <c r="F14" s="23" t="n"/>
       <c r="G14" s="23" t="n"/>
-      <c r="H14" s="23" t="inlineStr">
-        <is>
-          <t>ما تصمّم</t>
-        </is>
-      </c>
-      <c r="I14" s="22" t="inlineStr">
-        <is>
-          <t>اليوم 6</t>
-        </is>
-      </c>
+      <c r="H14" s="23" t="n"/>
+      <c r="I14" s="22" t="n"/>
     </row>
     <row r="15" ht="33.75" customHeight="1" s="16">
-      <c r="A15" s="23" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="21" t="n">
-        <v>46312</v>
-      </c>
-      <c r="C15" s="23" t="inlineStr">
-        <is>
-          <t>السبت</t>
-        </is>
-      </c>
-      <c r="D15" s="23" t="inlineStr">
-        <is>
-          <t>5:00 م</t>
-        </is>
-      </c>
-      <c r="E15" s="22" t="inlineStr">
-        <is>
-          <t>روبوت بسعر سيارة</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="inlineStr">
-        <is>
-          <t>كاروسل</t>
-        </is>
-      </c>
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="23" t="n"/>
+      <c r="D15" s="23" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="23" t="n"/>
       <c r="G15" s="23" t="n"/>
-      <c r="H15" s="23" t="inlineStr">
-        <is>
-          <t>ما تصمّم</t>
-        </is>
-      </c>
-      <c r="I15" s="22" t="inlineStr">
-        <is>
-          <t>اليوم 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17"/>
+      <c r="H15" s="23" t="n"/>
+      <c r="I15" s="22" t="n"/>
+    </row>
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="E18" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly carousel and reel #1 published; tracker updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -832,25 +832,53 @@
       </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
-          <t>جاهز</t>
+          <t>منشور</t>
         </is>
       </c>
       <c r="I9" s="24" t="inlineStr">
         <is>
-          <t>زياد ينشره يدويًا 5 العصر (15 شريحة أكثر من حد النشر التلقائي). صفحة الروابط في البايو.</t>
+          <t>نزل يدويًا 12:39 الظهر: https://www.instagram.com/p/DeY0xfwCusY/</t>
         </is>
       </c>
     </row>
     <row r="10" ht="33.75" customHeight="1" s="16">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="21" t="n"/>
-      <c r="C10" s="23" t="n"/>
-      <c r="D10" s="23" t="n"/>
-      <c r="E10" s="22" t="n"/>
-      <c r="F10" s="23" t="n"/>
+      <c r="A10" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>6:23 م</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>ريل ملخص أسبوع الذكاء الاصطناعي (العدد 1)</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>ريل</t>
+        </is>
+      </c>
       <c r="G10" s="23" t="n"/>
-      <c r="H10" s="23" t="n"/>
-      <c r="I10" s="22" t="n"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>منشور</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>نزل يدويًا بموسيقى من إنستقرام: https://www.instagram.com/reel/DeZb9q2KydT/</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="33.75" customHeight="1" s="16">
       <c r="A11" s="23" t="n"/>

</xml_diff>

<commit_message>
Student carousel moved to 13 Oct; Claude Design carousel rated bad (rejected); tracker updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -613,7 +613,7 @@
     <row r="2" ht="15" customHeight="1" s="16">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>آخر تحديث: 12 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
+          <t>آخر تحديث: 13 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
         </is>
       </c>
     </row>
@@ -881,26 +881,76 @@
       </c>
     </row>
     <row r="11" ht="33.75" customHeight="1" s="16">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="23" t="n"/>
-      <c r="E11" s="22" t="n"/>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="23" t="n"/>
-      <c r="H11" s="23" t="n"/>
-      <c r="I11" s="22" t="n"/>
+      <c r="A11" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E11" s="22" t="inlineStr">
+        <is>
+          <t>طالب جامعة؟ 4 أدوات ذكاء اصطناعي ببلاش</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>نشر تلقائي 5 العصر. الكلمة: «أدوات»</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="33.75" customHeight="1" s="16">
-      <c r="A12" s="23" t="n"/>
+      <c r="A12" s="23" t="n">
+        <v>8</v>
+      </c>
       <c r="B12" s="21" t="n"/>
       <c r="C12" s="23" t="n"/>
       <c r="D12" s="23" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="23" t="n"/>
-      <c r="G12" s="23" t="n"/>
-      <c r="H12" s="23" t="n"/>
-      <c r="I12" s="22" t="n"/>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>كيف تستخدم كلود في التصميم</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>سيئ</t>
+        </is>
+      </c>
+      <c r="I12" s="22" t="inlineStr">
+        <is>
+          <t>زياد قيّمه سيئ: مو المطلوب. ما بينزل.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="33.75" customHeight="1" s="16">
       <c r="A13" s="23" t="n"/>
@@ -1036,7 +1086,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="H5:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>"منشور,مجدول,جاهز,قيد التصميم,ما تصمّم"</formula1>
+      <formula1>"منشور,مجدول,جاهز,قيد التصميم,ما تصمّم,سيئ"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish student tools carousel (13 Oct, 17:02 Muscat)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -617,6 +617,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="16">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -912,12 +913,12 @@
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>مجدول</t>
+          <t>منشور</t>
         </is>
       </c>
       <c r="I11" s="22" t="inlineStr">
         <is>
-          <t>نشر تلقائي 5 العصر. الكلمة: «أدوات»</t>
+          <t>نُشر 5:02 العصر. https://www.instagram.com/p/Deb3rqloAe6/ الكلمة: «أدوات» (رد تلقائي يوجّه لرابط البايو)</t>
         </is>
       </c>
     </row>
@@ -985,6 +986,8 @@
       <c r="H15" s="23" t="n"/>
       <c r="I15" s="22" t="n"/>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="E18" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
AI zone carousel: post.json pinned to 0bff8fc, scheduled 16 Oct 17:00 Muscat (test container FINISHED)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -613,11 +613,10 @@
     <row r="2" ht="15" customHeight="1" s="16">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>آخر تحديث: 13 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>آخر تحديث: 16 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="30" customHeight="1" s="16">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -954,15 +953,45 @@
       </c>
     </row>
     <row r="13" ht="33.75" customHeight="1" s="16">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="23" t="n"/>
-      <c r="D13" s="23" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="23" t="n"/>
-      <c r="G13" s="23" t="n"/>
-      <c r="H13" s="23" t="n"/>
-      <c r="I13" s="22" t="n"/>
+      <c r="A13" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>مايكروسوفت وآي بي إم يتباحثون مع شركة عمانية (منطقة الذكاء الاصطناعي)</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>صور حقيقية، والصفحة الأخيرة فيها الحساب ودعوة للمتابعة. مجدول 5 العصر.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="33.75" customHeight="1" s="16">
       <c r="A14" s="23" t="n"/>
@@ -986,8 +1015,6 @@
       <c r="H15" s="23" t="n"/>
       <c r="I15" s="22" t="n"/>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="E18" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Publish AI zone carousel (16 Oct, 15:07 Muscat)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KfNMA3U7kT2oyRtTnKGRw8
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="15" min="1" max="1"/>
@@ -966,7 +966,7 @@
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>5:00 م</t>
+          <t>3:07 م</t>
         </is>
       </c>
       <c r="E13" s="22" t="inlineStr">
@@ -984,12 +984,12 @@
       </c>
       <c r="H13" s="23" t="inlineStr">
         <is>
-          <t>مجدول</t>
+          <t>منشور</t>
         </is>
       </c>
       <c r="I13" s="22" t="inlineStr">
         <is>
-          <t>صور حقيقية، والصفحة الأخيرة فيها الحساب ودعوة للمتابعة. مجدول 5 العصر.</t>
+          <t>نزل 3:07 العصر بطلب زياد («الحين»): https://www.instagram.com/p/DejY4NnFfHp/</t>
         </is>
       </c>
     </row>
@@ -1015,6 +1015,8 @@
       <c r="H15" s="23" t="n"/>
       <c r="I15" s="22" t="n"/>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="E18" s="25" t="inlineStr">
         <is>
@@ -1095,6 +1097,16 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
   </sheetData>
   <autoFilter ref="A4:I15"/>
   <conditionalFormatting sqref="A5:I35">

</xml_diff>

<commit_message>
Tracker: Claude series rows, first carousel published
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -613,7 +613,7 @@
     <row r="2" ht="15" customHeight="1" s="16">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>آخر تحديث: 16 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
+          <t>آخر تحديث: 23 أكتوبر 2026 · وقت النشر موحّد الساعة 5 العصر كل يوم · عدّل عمود "الحالة" من القائمة، واكتب ملاحظاتك في عمود "ملاحظات".</t>
         </is>
       </c>
     </row>
@@ -994,121 +994,381 @@
       </c>
     </row>
     <row r="14" ht="33.75" customHeight="1" s="16">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="23" t="n"/>
-      <c r="D14" s="23" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="23" t="n"/>
-      <c r="G14" s="23" t="n"/>
-      <c r="H14" s="23" t="n"/>
-      <c r="I14" s="22" t="n"/>
+      <c r="A14" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>12:10 ص</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>سلسلة كلود: لا تستخدم كلود قبل ما تسوي هالشي (التعليمات، الذاكرة، النموذج، المحادثة المخفية)</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G14" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>منشور</t>
+        </is>
+      </c>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>نزل 12:10 الفجر بطلب زياد («الحين»): https://www.instagram.com/p/Dezzu6knQmC/ · ثيم فاتح ولقطات حقيقية من حسابه</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="33.75" customHeight="1" s="16">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="23" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="23" t="n"/>
-      <c r="G15" s="23" t="n"/>
-      <c r="H15" s="23" t="n"/>
-      <c r="I15" s="22" t="n"/>
-    </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18" ht="15" customHeight="1" s="16">
-      <c r="E18" s="25" t="inlineStr">
+      <c r="A15" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>سلسلة كلود: كلّمه (قواعد أنثروبيك بأمثلة قبل وبعد)</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>ما تصمّم</t>
+        </is>
+      </c>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>الهوك المقترح: «أنثروبيك نفسها تقولك كيف تكلّم كلود»</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="33.75" customHeight="1" s="16">
+      <c r="A16" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>46320</v>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>سلسلة كلود: نظّمه (المشاريع: ملفات وتعليمات مرة وحدة)</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>ما تصمّم</t>
+        </is>
+      </c>
+      <c r="I16" s="22" t="inlineStr">
+        <is>
+          <t>الهوك المقترح: «لا تشرح لكلود نفس الشي كل مرة». تعليمات المشروع في المجاني تنتأكد من التطبيق</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="33.75" customHeight="1" s="16">
+      <c r="A17" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>سلسلة كلود: ملفاتك (يقرأ PDF والصور ويسلّمك إكسل ووورد وعرض)</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>ما تصمّم</t>
+        </is>
+      </c>
+      <c r="I17" s="22" t="inlineStr">
+        <is>
+          <t>الهوك المقترح: «كلود يسلّمك ملف إكسل جاهز.. ببلاش»</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="33.75" customHeight="1" s="16">
+      <c r="A18" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>46322</v>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>سلسلة كلود: اربطه (Gmail والتقويم وDrive)</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>ما تصمّم</t>
+        </is>
+      </c>
+      <c r="I18" s="22" t="inlineStr">
+        <is>
+          <t>الهوك المقترح: «خلّ كلود يقرأ إيميلك بدالك»</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="33.75" customHeight="1" s="16">
+      <c r="A19" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>46323</v>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>سلسلة كلود: تأكد واحمِ نفسك (المصادر، البيانات الحساسة، إعداد التدريب)</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>ما تصمّم</t>
+        </is>
+      </c>
+      <c r="I19" s="22" t="inlineStr">
+        <is>
+          <t>الهوك المقترح: «أنثروبيك تقولك: لا تصدق كلود دايم»</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="33.75" customHeight="1" s="16">
+      <c r="A20" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>46324</v>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>5:00 م</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>سلسلة كلود: وفّر حدودك + خريطة الأسبوع</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>ما تصمّم</t>
+        </is>
+      </c>
+      <c r="I20" s="22" t="inlineStr">
+        <is>
+          <t>الهوك المقترح: «للحين يطلع لك "وصلت الحد" في كلود؟». الكلمة: «كلود» (دليل كامل)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23" ht="15" customHeight="1" s="16">
+      <c r="E23" s="25" t="inlineStr">
         <is>
           <t>ملخص الحالة</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="16">
-      <c r="E19" s="26" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="16">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>منشور</t>
         </is>
       </c>
-      <c r="F19" s="27">
-        <f>COUNTIF($H$5:$H$35,E19)</f>
+      <c r="F24" s="27">
+        <f>COUNTIF($H$5:$H$35,E24)</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="16">
-      <c r="E20" s="26" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="16">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>مجدول</t>
         </is>
       </c>
-      <c r="F20" s="27">
-        <f>COUNTIF($H$5:$H$35,E20)</f>
+      <c r="F25" s="27">
+        <f>COUNTIF($H$5:$H$35,E25)</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="16">
-      <c r="E21" s="26" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="16">
+      <c r="E26" s="26" t="inlineStr">
         <is>
           <t>جاهز</t>
         </is>
       </c>
-      <c r="F21" s="27">
-        <f>COUNTIF($H$5:$H$35,E21)</f>
+      <c r="F26" s="27">
+        <f>COUNTIF($H$5:$H$35,E26)</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="16">
-      <c r="E22" s="26" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="16">
+      <c r="E27" s="26" t="inlineStr">
         <is>
           <t>قيد التصميم</t>
         </is>
       </c>
-      <c r="F22" s="27">
-        <f>COUNTIF($H$5:$H$35,E22)</f>
+      <c r="F27" s="27">
+        <f>COUNTIF($H$5:$H$35,E27)</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="16">
-      <c r="E23" s="26" t="inlineStr">
+    <row r="28" ht="15" customHeight="1" s="16">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>ما تصمّم</t>
         </is>
       </c>
-      <c r="F23" s="27">
-        <f>COUNTIF($H$5:$H$35,E23)</f>
+      <c r="F28" s="27">
+        <f>COUNTIF($H$5:$H$35,E28)</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="16">
-      <c r="E24" s="28" t="inlineStr">
+    <row r="29" ht="15" customHeight="1" s="16">
+      <c r="E29" s="28" t="inlineStr">
         <is>
           <t>المجموع</t>
         </is>
       </c>
-      <c r="F24" s="29">
-        <f>SUM(F19:F23)</f>
+      <c r="F29" s="29">
+        <f>SUM(F24:F28)</f>
         <v/>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="16">
-      <c r="E25" s="30" t="inlineStr">
+    <row r="30" ht="15" customHeight="1" s="16">
+      <c r="E30" s="30" t="inlineStr">
         <is>
           <t>العدّ يشمل الصفوف من 5 إلى 35، فأي صف جديد تضيفه تحت الجدول ينحسب تلقائيًا.</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31"/>
     <row r="32"/>
     <row r="33"/>
     <row r="34"/>
     <row r="35"/>
   </sheetData>
-  <autoFilter ref="A4:I15"/>
+  <autoFilter ref="A4:I20"/>
   <conditionalFormatting sqref="A5:I35">
     <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="7" text="" percent="0" bottom="0">
       <formula>$H5="منشور"</formula>

</xml_diff>

<commit_message>
Tracker: Claude prompting carousel scheduled Fri 11:00
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -1039,21 +1039,21 @@
         <v>11</v>
       </c>
       <c r="B15" s="21" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>السبت</t>
+          <t>الجمعة</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>5:00 م</t>
+          <t>11:00 ص</t>
         </is>
       </c>
       <c r="E15" s="22" t="inlineStr">
         <is>
-          <t>سلسلة كلود: كلّمه (قواعد أنثروبيك بأمثلة قبل وبعد)</t>
+          <t>سلسلة كلود: انت تكلّم كلود غلط (قواعد أنثروبيك بمثال رسالة الإجازة)</t>
         </is>
       </c>
       <c r="F15" s="23" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="H15" s="23" t="inlineStr">
         <is>
-          <t>ما تصمّم</t>
+          <t>مجدول</t>
         </is>
       </c>
       <c r="I15" s="22" t="inlineStr">
         <is>
-          <t>الهوك المقترح: «أنثروبيك نفسها تقولك كيف تكلّم كلود»</t>
+          <t>مجدول 11 الصبح بطلب زياد · المسودة 18498461098100078 · الصور على commit 0d02749 · براند زياد في الغلاف والفوتر</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: Claude + Gmail carousel scheduled Fri 11:00
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -1038,17 +1038,15 @@
       <c r="A15" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="21" t="n">
-        <v>46318</v>
-      </c>
+      <c r="B15" s="21" t="n"/>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>الجمعة</t>
+          <t/>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>11:00 ص</t>
+          <t/>
         </is>
       </c>
       <c r="E15" s="22" t="inlineStr">
@@ -1066,12 +1064,12 @@
       </c>
       <c r="H15" s="23" t="inlineStr">
         <is>
-          <t>مجدول</t>
+          <t>جاهز</t>
         </is>
       </c>
       <c r="I15" s="22" t="inlineStr">
         <is>
-          <t>مجدول 11 الصبح بطلب زياد · المسودة 18498461098100078 · الصور على commit 0d02749 · براند زياد في الغلاف والفوتر</t>
+          <t>جاهز ومرفوع (commit 0d02749). ما انجدول: زياد اختار «كلود والإيميل» للجمعة. المسودة القديمة تنتهي خلال 24 ساعة</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1278,47 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
+    <row r="21" ht="33.75" customHeight="1" s="16">
+      <c r="A21" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>11:00 ص</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>كلود صار يرد على إيميلاتك… بس بإذنك (ربط جيميل)</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>كاروسل</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+      <c r="I21" s="22" t="inlineStr">
+        <is>
+          <t>مجدول 11 الصبح بطلب زياد · المسودة 18498462697100078 · الصور على commit 0e14ba7 · حسابه في الفوتر وصورته في الأخيرة</t>
+        </is>
+      </c>
+    </row>
     <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="16">
       <c r="E23" s="25" t="inlineStr">
@@ -1368,7 +1406,7 @@
     <row r="34"/>
     <row r="35"/>
   </sheetData>
-  <autoFilter ref="A4:I20"/>
+  <autoFilter ref="A4:I21"/>
   <conditionalFormatting sqref="A5:I35">
     <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="7" text="" percent="0" bottom="0">
       <formula>$H5="منشور"</formula>

</xml_diff>

<commit_message>
Tracker: Claude + Gmail carousel published
</commit_message>
<xml_diff>
--- a/plan/ziyad-content-schedule.xlsx
+++ b/plan/ziyad-content-schedule.xlsx
@@ -1292,7 +1292,7 @@
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>11:00 ص</t>
+          <t>7:03 م</t>
         </is>
       </c>
       <c r="E21" s="22" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="H21" s="23" t="inlineStr">
         <is>
-          <t>مجدول</t>
+          <t>منشور</t>
         </is>
       </c>
       <c r="I21" s="22" t="inlineStr">
         <is>
-          <t>مجدول 11 الصبح بطلب زياد · المسودة 18498462697100078 · الصور على commit 0e14ba7 · حسابه في الفوتر وصورته في الأخيرة</t>
+          <t>نزل 7:03 مساء بطلب زياد («نزله الحين»): https://www.instagram.com/p/De11aXiIFy-/ · موعد 11 الصبح ما مشى (Composio ما رد) · تصميم جديد بترتيب بوست الشحن وخط Tajawal · الصور على commit 1015045</t>
         </is>
       </c>
     </row>

</xml_diff>